<commit_message>
[Fixing, fixed] Fixing regex Lazada Tax inv address issue, fixed dtype issue
[Fixing] Lazada Tax inv address issue,
[Fixed] Data type some fields of lazada's dataframe
</commit_message>
<xml_diff>
--- a/output_test.xlsx
+++ b/output_test.xlsx
@@ -761,7 +761,8 @@
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>603565000061.0</t>
+          <t xml:space="preserve">0603565000061
+</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
@@ -981,7 +982,7 @@
       </c>
       <c r="W5" t="inlineStr">
         <is>
-          <t>1027243678.0</t>
+          <t>1027243678</t>
         </is>
       </c>
       <c r="X5" t="inlineStr">
@@ -1301,7 +1302,7 @@
       </c>
       <c r="W8" t="inlineStr">
         <is>
-          <t>653554001168.0</t>
+          <t>0653554001168</t>
         </is>
       </c>
       <c r="X8" t="inlineStr">
@@ -1413,7 +1414,7 @@
       </c>
       <c r="W9" t="inlineStr">
         <is>
-          <t>3901000219646.0</t>
+          <t>3901000219646</t>
         </is>
       </c>
       <c r="X9" t="inlineStr">
@@ -2153,7 +2154,7 @@
       </c>
       <c r="W16" t="inlineStr">
         <is>
-          <t>3600700003397.0</t>
+          <t>3600700003397</t>
         </is>
       </c>
       <c r="X16" t="inlineStr">
@@ -2265,7 +2266,7 @@
       </c>
       <c r="W17" t="inlineStr">
         <is>
-          <t>1100400631595.0</t>
+          <t>1100400631595</t>
         </is>
       </c>
       <c r="X17" t="inlineStr">

</xml_diff>

<commit_message>
patch: compatibilityกับ pandas ver3.0
pandas อัพเดท lib ใหม่เป็น ver3 ณ ปัจจุบันในproject ใช้ 2.2 ทำให้ warning วีธีการเรียกหาค่าใน column เนื่องจาก ver3 จะมองวิธีการหา column แบบเดิมได้แต่รเข้าใจว่า logic ไม่ชัดเจน เลยปรับใหม่ให้ชัดเจนสำหรับ ver3 จริงๆก็ใช้ 2.2 ได้แหละ แต่เผื่อไว้ก่อน เผื่อมันวกกลับมา ver เดิมไม่ได้
</commit_message>
<xml_diff>
--- a/output_test.xlsx
+++ b/output_test.xlsx
@@ -16,7 +16,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
+  </numFmts>
   <fonts count="2">
     <font>
       <name val="Calibri"/>
@@ -55,11 +58,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -687,10 +691,8 @@
       <c r="Z2" t="n">
         <v>3265</v>
       </c>
-      <c r="AA2" t="inlineStr">
-        <is>
-          <t>2026-04-16 00:36</t>
-        </is>
+      <c r="AA2" s="2" t="n">
+        <v>46128.025</v>
       </c>
       <c r="AB2" t="inlineStr"/>
       <c r="AC2" t="n">
@@ -805,10 +807,8 @@
       <c r="Z3" t="n">
         <v>5302.5</v>
       </c>
-      <c r="AA3" t="inlineStr">
-        <is>
-          <t>2026-04-16 07:02</t>
-        </is>
+      <c r="AA3" s="2" t="n">
+        <v>46128.29305555556</v>
       </c>
       <c r="AB3" t="inlineStr"/>
       <c r="AC3" t="n">
@@ -923,10 +923,8 @@
       <c r="Z4" t="n">
         <v>5088.75</v>
       </c>
-      <c r="AA4" t="inlineStr">
-        <is>
-          <t>2026-04-16 07:49</t>
-        </is>
+      <c r="AA4" s="2" t="n">
+        <v>46128.32569444444</v>
       </c>
       <c r="AB4" t="inlineStr"/>
       <c r="AC4" t="n">
@@ -1049,10 +1047,8 @@
       <c r="Z5" t="n">
         <v>4620</v>
       </c>
-      <c r="AA5" t="inlineStr">
-        <is>
-          <t>2026-04-16 09:29</t>
-        </is>
+      <c r="AA5" s="2" t="n">
+        <v>46128.39513888889</v>
       </c>
       <c r="AB5" t="inlineStr"/>
       <c r="AC5" t="n">
@@ -1167,10 +1163,8 @@
       <c r="Z6" t="n">
         <v>6427</v>
       </c>
-      <c r="AA6" t="inlineStr">
-        <is>
-          <t>2026-04-16 10:11</t>
-        </is>
+      <c r="AA6" s="2" t="n">
+        <v>46128.42430555556</v>
       </c>
       <c r="AB6" t="inlineStr"/>
       <c r="AC6" t="n">
@@ -1285,10 +1279,8 @@
       <c r="Z7" t="n">
         <v>1399</v>
       </c>
-      <c r="AA7" t="inlineStr">
-        <is>
-          <t>2026-04-16 10:42</t>
-        </is>
+      <c r="AA7" s="2" t="n">
+        <v>46128.44583333333</v>
       </c>
       <c r="AB7" t="inlineStr"/>
       <c r="AC7" t="n">
@@ -1407,10 +1399,8 @@
       <c r="Z8" t="n">
         <v>6087.75</v>
       </c>
-      <c r="AA8" t="inlineStr">
-        <is>
-          <t>2026-04-16 13:48</t>
-        </is>
+      <c r="AA8" s="2" t="n">
+        <v>46128.575</v>
       </c>
       <c r="AB8" t="inlineStr"/>
       <c r="AC8" t="n">
@@ -1533,10 +1523,8 @@
       <c r="Z9" t="n">
         <v>4350.5</v>
       </c>
-      <c r="AA9" t="inlineStr">
-        <is>
-          <t>2026-04-16 21:17</t>
-        </is>
+      <c r="AA9" s="2" t="n">
+        <v>46128.88680555556</v>
       </c>
       <c r="AB9" t="inlineStr"/>
       <c r="AC9" t="n">
@@ -1651,10 +1639,8 @@
       <c r="Z10" t="n">
         <v>1075.5</v>
       </c>
-      <c r="AA10" t="inlineStr">
-        <is>
-          <t>2026-04-16 22:34</t>
-        </is>
+      <c r="AA10" s="2" t="n">
+        <v>46128.94027777778</v>
       </c>
       <c r="AB10" t="inlineStr"/>
       <c r="AC10" t="n">
@@ -1773,10 +1759,8 @@
       <c r="Z11" t="n">
         <v>1188</v>
       </c>
-      <c r="AA11" t="inlineStr">
-        <is>
-          <t>2026-04-17 08:48</t>
-        </is>
+      <c r="AA11" s="2" t="n">
+        <v>46129.36666666667</v>
       </c>
       <c r="AB11" t="inlineStr"/>
       <c r="AC11" t="n">
@@ -1895,10 +1879,8 @@
       <c r="Z12" t="n">
         <v>1188</v>
       </c>
-      <c r="AA12" t="inlineStr">
-        <is>
-          <t>2026-04-17 08:45</t>
-        </is>
+      <c r="AA12" s="2" t="n">
+        <v>46129.36458333334</v>
       </c>
       <c r="AB12" t="inlineStr"/>
       <c r="AC12" t="n">
@@ -2017,10 +1999,8 @@
       <c r="Z13" t="n">
         <v>896.03</v>
       </c>
-      <c r="AA13" t="inlineStr">
-        <is>
-          <t>2026-04-17 11:48</t>
-        </is>
+      <c r="AA13" s="2" t="n">
+        <v>46129.49166666667</v>
       </c>
       <c r="AB13" t="inlineStr"/>
       <c r="AC13" t="n">
@@ -2135,10 +2115,8 @@
       <c r="Z14" t="n">
         <v>1850.25</v>
       </c>
-      <c r="AA14" t="inlineStr">
-        <is>
-          <t>2026-04-17 12:51</t>
-        </is>
+      <c r="AA14" s="2" t="n">
+        <v>46129.53541666667</v>
       </c>
       <c r="AB14" t="inlineStr"/>
       <c r="AC14" t="n">
@@ -2253,10 +2231,8 @@
       <c r="Z15" t="n">
         <v>1850.25</v>
       </c>
-      <c r="AA15" t="inlineStr">
-        <is>
-          <t>2026-04-17 12:51</t>
-        </is>
+      <c r="AA15" s="2" t="n">
+        <v>46129.53541666667</v>
       </c>
       <c r="AB15" t="inlineStr"/>
       <c r="AC15" t="n">
@@ -2375,10 +2351,8 @@
       <c r="Z16" t="n">
         <v>756.6</v>
       </c>
-      <c r="AA16" t="inlineStr">
-        <is>
-          <t>2026-04-17 14:45</t>
-        </is>
+      <c r="AA16" s="2" t="n">
+        <v>46129.61458333334</v>
       </c>
       <c r="AB16" t="inlineStr"/>
       <c r="AC16" t="n">
@@ -2501,10 +2475,8 @@
       <c r="Z17" t="n">
         <v>6530.25</v>
       </c>
-      <c r="AA17" t="inlineStr">
-        <is>
-          <t>2026-04-17 18:51</t>
-        </is>
+      <c r="AA17" s="2" t="n">
+        <v>46129.78541666667</v>
       </c>
       <c r="AB17" t="inlineStr"/>
       <c r="AC17" t="n">
@@ -2623,10 +2595,8 @@
       <c r="Z18" t="n">
         <v>6530.25</v>
       </c>
-      <c r="AA18" t="inlineStr">
-        <is>
-          <t>2026-04-17 18:51</t>
-        </is>
+      <c r="AA18" s="2" t="n">
+        <v>46129.78541666667</v>
       </c>
       <c r="AB18" t="inlineStr"/>
       <c r="AC18" t="n">
@@ -2745,10 +2715,8 @@
       <c r="Z19" t="n">
         <v>5415</v>
       </c>
-      <c r="AA19" t="inlineStr">
-        <is>
-          <t>2026-04-17 18:36</t>
-        </is>
+      <c r="AA19" s="2" t="n">
+        <v>46129.775</v>
       </c>
       <c r="AB19" t="inlineStr"/>
       <c r="AC19" t="n">
@@ -2867,10 +2835,8 @@
       <c r="Z20" t="n">
         <v>5865</v>
       </c>
-      <c r="AA20" t="inlineStr">
-        <is>
-          <t>2026-04-17 18:31</t>
-        </is>
+      <c r="AA20" s="2" t="n">
+        <v>46129.77152777778</v>
       </c>
       <c r="AB20" t="inlineStr"/>
       <c r="AC20" t="n">
@@ -2985,10 +2951,8 @@
       <c r="Z21" t="n">
         <v>609</v>
       </c>
-      <c r="AA21" t="inlineStr">
-        <is>
-          <t>2026-04-18 12:34</t>
-        </is>
+      <c r="AA21" s="2" t="n">
+        <v>46130.52361111111</v>
       </c>
       <c r="AB21" t="inlineStr"/>
       <c r="AC21" t="n">
@@ -3103,10 +3067,8 @@
       <c r="Z22" t="n">
         <v>2254</v>
       </c>
-      <c r="AA22" t="inlineStr">
-        <is>
-          <t>2026-04-18 16:25</t>
-        </is>
+      <c r="AA22" s="2" t="n">
+        <v>46130.68402777778</v>
       </c>
       <c r="AB22" t="inlineStr"/>
       <c r="AC22" t="n">
@@ -3221,10 +3183,8 @@
       <c r="Z23" t="n">
         <v>1589</v>
       </c>
-      <c r="AA23" t="inlineStr">
-        <is>
-          <t>2026-04-18 17:16</t>
-        </is>
+      <c r="AA23" s="2" t="n">
+        <v>46130.71944444445</v>
       </c>
       <c r="AB23" t="inlineStr"/>
       <c r="AC23" t="n">
@@ -3339,10 +3299,8 @@
       <c r="Z24" t="n">
         <v>4184</v>
       </c>
-      <c r="AA24" t="inlineStr">
-        <is>
-          <t>2026-04-18 20:38</t>
-        </is>
+      <c r="AA24" s="2" t="n">
+        <v>46130.85972222222</v>
       </c>
       <c r="AB24" t="inlineStr"/>
       <c r="AC24" t="n">
@@ -3461,10 +3419,8 @@
       <c r="Z25" t="n">
         <v>498.61</v>
       </c>
-      <c r="AA25" t="inlineStr">
-        <is>
-          <t>2026-04-18 21:41</t>
-        </is>
+      <c r="AA25" s="2" t="n">
+        <v>46130.90347222222</v>
       </c>
       <c r="AB25" t="inlineStr"/>
       <c r="AC25" t="n">
@@ -3583,10 +3539,8 @@
       <c r="Z26" t="n">
         <v>25634</v>
       </c>
-      <c r="AA26" t="inlineStr">
-        <is>
-          <t>2026-04-18 21:42</t>
-        </is>
+      <c r="AA26" s="2" t="n">
+        <v>46130.90416666667</v>
       </c>
       <c r="AB26" t="inlineStr"/>
       <c r="AC26" t="n">
@@ -3709,10 +3663,8 @@
       <c r="Z27" t="n">
         <v>23947</v>
       </c>
-      <c r="AA27" t="inlineStr">
-        <is>
-          <t>2026-04-19 11:56</t>
-        </is>
+      <c r="AA27" s="2" t="n">
+        <v>46131.49722222222</v>
       </c>
       <c r="AB27" t="inlineStr"/>
       <c r="AC27" t="n">
@@ -3835,10 +3787,8 @@
       <c r="Z28" t="n">
         <v>5652</v>
       </c>
-      <c r="AA28" t="inlineStr">
-        <is>
-          <t>2026-04-19 13:24</t>
-        </is>
+      <c r="AA28" s="2" t="n">
+        <v>46131.55833333333</v>
       </c>
       <c r="AB28" t="inlineStr"/>
       <c r="AC28" t="n">
@@ -3961,10 +3911,8 @@
       <c r="Z29" t="n">
         <v>744</v>
       </c>
-      <c r="AA29" t="inlineStr">
-        <is>
-          <t>2026-04-19 14:57</t>
-        </is>
+      <c r="AA29" s="2" t="n">
+        <v>46131.62291666667</v>
       </c>
       <c r="AB29" t="inlineStr"/>
       <c r="AC29" t="n">
@@ -4087,10 +4035,8 @@
       <c r="Z30" t="n">
         <v>744</v>
       </c>
-      <c r="AA30" t="inlineStr">
-        <is>
-          <t>2026-04-19 14:57</t>
-        </is>
+      <c r="AA30" s="2" t="n">
+        <v>46131.62291666667</v>
       </c>
       <c r="AB30" t="inlineStr"/>
       <c r="AC30" t="n">
@@ -4209,10 +4155,8 @@
       <c r="Z31" t="n">
         <v>1187</v>
       </c>
-      <c r="AA31" t="inlineStr">
-        <is>
-          <t>2026-04-19 16:17</t>
-        </is>
+      <c r="AA31" s="2" t="n">
+        <v>46131.67847222222</v>
       </c>
       <c r="AB31" t="inlineStr"/>
       <c r="AC31" t="n">
@@ -4331,10 +4275,8 @@
       <c r="Z32" t="n">
         <v>1187</v>
       </c>
-      <c r="AA32" t="inlineStr">
-        <is>
-          <t>2026-04-19 16:17</t>
-        </is>
+      <c r="AA32" s="2" t="n">
+        <v>46131.67847222222</v>
       </c>
       <c r="AB32" t="inlineStr"/>
       <c r="AC32" t="n">
@@ -4449,10 +4391,8 @@
       <c r="Z33" t="n">
         <v>6019</v>
       </c>
-      <c r="AA33" t="inlineStr">
-        <is>
-          <t>2026-04-19 16:49</t>
-        </is>
+      <c r="AA33" s="2" t="n">
+        <v>46131.70069444444</v>
       </c>
       <c r="AB33" t="inlineStr"/>
       <c r="AC33" t="n">
@@ -4571,10 +4511,8 @@
       <c r="Z34" t="n">
         <v>1123</v>
       </c>
-      <c r="AA34" t="inlineStr">
-        <is>
-          <t>2026-04-19 16:25</t>
-        </is>
+      <c r="AA34" s="2" t="n">
+        <v>46131.68402777778</v>
       </c>
       <c r="AB34" t="inlineStr"/>
       <c r="AC34" t="n">
@@ -4697,10 +4635,8 @@
       <c r="Z35" t="n">
         <v>1123</v>
       </c>
-      <c r="AA35" t="inlineStr">
-        <is>
-          <t>2026-04-19 16:25</t>
-        </is>
+      <c r="AA35" s="2" t="n">
+        <v>46131.68402777778</v>
       </c>
       <c r="AB35" t="inlineStr"/>
       <c r="AC35" t="n">
@@ -4815,10 +4751,8 @@
       <c r="Z36" t="n">
         <v>308</v>
       </c>
-      <c r="AA36" t="inlineStr">
-        <is>
-          <t>2026-04-19 21:49</t>
-        </is>
+      <c r="AA36" s="2" t="n">
+        <v>46131.90902777778</v>
       </c>
       <c r="AB36" t="inlineStr"/>
       <c r="AC36" t="n">
@@ -4937,10 +4871,8 @@
       <c r="Z37" t="n">
         <v>492</v>
       </c>
-      <c r="AA37" t="inlineStr">
-        <is>
-          <t>2026-04-20 09:52</t>
-        </is>
+      <c r="AA37" s="2" t="n">
+        <v>46132.41111111111</v>
       </c>
       <c r="AB37" t="inlineStr"/>
       <c r="AC37" t="n">
@@ -5059,10 +4991,8 @@
       <c r="Z38" t="n">
         <v>12640</v>
       </c>
-      <c r="AA38" t="inlineStr">
-        <is>
-          <t>2026-04-20 10:39</t>
-        </is>
+      <c r="AA38" s="2" t="n">
+        <v>46132.44375</v>
       </c>
       <c r="AB38" t="inlineStr"/>
       <c r="AC38" t="n">
@@ -5177,10 +5107,8 @@
       <c r="Z39" t="n">
         <v>2212</v>
       </c>
-      <c r="AA39" t="inlineStr">
-        <is>
-          <t>2026-04-20 11:20</t>
-        </is>
+      <c r="AA39" s="2" t="n">
+        <v>46132.47222222222</v>
       </c>
       <c r="AB39" t="inlineStr"/>
       <c r="AC39" t="n">
@@ -5299,10 +5227,8 @@
       <c r="Z40" t="n">
         <v>20852</v>
       </c>
-      <c r="AA40" t="inlineStr">
-        <is>
-          <t>2026-04-20 16:19</t>
-        </is>
+      <c r="AA40" s="2" t="n">
+        <v>46132.67986111111</v>
       </c>
       <c r="AB40" t="inlineStr"/>
       <c r="AC40" t="n">
@@ -5421,10 +5347,8 @@
       <c r="Z41" t="n">
         <v>178</v>
       </c>
-      <c r="AA41" t="inlineStr">
-        <is>
-          <t>2026-04-20 18:10</t>
-        </is>
+      <c r="AA41" s="2" t="n">
+        <v>46132.75694444445</v>
       </c>
       <c r="AB41" t="inlineStr"/>
       <c r="AC41" t="n">
@@ -5539,10 +5463,8 @@
       <c r="Z42" t="n">
         <v>406.85</v>
       </c>
-      <c r="AA42" t="inlineStr">
-        <is>
-          <t>2026-04-20 21:05</t>
-        </is>
+      <c r="AA42" s="2" t="n">
+        <v>46132.87847222222</v>
       </c>
       <c r="AB42" t="inlineStr"/>
       <c r="AC42" t="n">
@@ -5661,10 +5583,8 @@
       <c r="Z43" t="n">
         <v>3070.08</v>
       </c>
-      <c r="AA43" t="inlineStr">
-        <is>
-          <t>2026-04-20 21:48</t>
-        </is>
+      <c r="AA43" s="2" t="n">
+        <v>46132.90833333333</v>
       </c>
       <c r="AB43" t="inlineStr"/>
       <c r="AC43" t="n">
@@ -5779,10 +5699,8 @@
       <c r="Z44" t="n">
         <v>2010</v>
       </c>
-      <c r="AA44" t="inlineStr">
-        <is>
-          <t>2026-04-20 22:36</t>
-        </is>
+      <c r="AA44" s="2" t="n">
+        <v>46132.94166666667</v>
       </c>
       <c r="AB44" t="inlineStr"/>
       <c r="AC44" t="n">
@@ -5901,10 +5819,8 @@
       <c r="Z45" t="n">
         <v>574</v>
       </c>
-      <c r="AA45" t="inlineStr">
-        <is>
-          <t>2026-04-21 11:01</t>
-        </is>
+      <c r="AA45" s="2" t="n">
+        <v>46133.45902777778</v>
       </c>
       <c r="AB45" t="inlineStr"/>
       <c r="AC45" t="n">
@@ -6019,10 +5935,8 @@
       <c r="Z46" t="n">
         <v>5793</v>
       </c>
-      <c r="AA46" t="inlineStr">
-        <is>
-          <t>2026-04-21 12:45</t>
-        </is>
+      <c r="AA46" s="2" t="n">
+        <v>46133.53125</v>
       </c>
       <c r="AB46" t="inlineStr"/>
       <c r="AC46" t="n">
@@ -6137,10 +6051,8 @@
       <c r="Z47" t="n">
         <v>4145</v>
       </c>
-      <c r="AA47" t="inlineStr">
-        <is>
-          <t>2026-04-21 17:56</t>
-        </is>
+      <c r="AA47" s="2" t="n">
+        <v>46133.74722222222</v>
       </c>
       <c r="AB47" t="inlineStr"/>
       <c r="AC47" t="n">
@@ -6259,10 +6171,8 @@
       <c r="Z48" t="n">
         <v>4693</v>
       </c>
-      <c r="AA48" t="inlineStr">
-        <is>
-          <t>2026-04-21 17:36</t>
-        </is>
+      <c r="AA48" s="2" t="n">
+        <v>46133.73333333333</v>
       </c>
       <c r="AB48" t="inlineStr"/>
       <c r="AC48" t="n">
@@ -6377,10 +6287,8 @@
       <c r="Z49" t="n">
         <v>27674</v>
       </c>
-      <c r="AA49" t="inlineStr">
-        <is>
-          <t>2026-04-21 21:07</t>
-        </is>
+      <c r="AA49" s="2" t="n">
+        <v>46133.87986111111</v>
       </c>
       <c r="AB49" t="inlineStr"/>
       <c r="AC49" t="n">
@@ -6499,10 +6407,8 @@
       <c r="Z50" t="n">
         <v>1013</v>
       </c>
-      <c r="AA50" t="inlineStr">
-        <is>
-          <t>2026-04-22 14:53</t>
-        </is>
+      <c r="AA50" s="2" t="n">
+        <v>46134.62013888889</v>
       </c>
       <c r="AB50" t="inlineStr"/>
       <c r="AC50" t="n">
@@ -6621,10 +6527,8 @@
       <c r="Z51" t="n">
         <v>1179</v>
       </c>
-      <c r="AA51" t="inlineStr">
-        <is>
-          <t>2026-04-22 17:17</t>
-        </is>
+      <c r="AA51" s="2" t="n">
+        <v>46134.72013888889</v>
       </c>
       <c r="AB51" t="inlineStr"/>
       <c r="AC51" t="n">
@@ -6743,10 +6647,8 @@
       <c r="Z52" t="n">
         <v>2023.25</v>
       </c>
-      <c r="AA52" t="inlineStr">
-        <is>
-          <t>2026-04-16 01:36</t>
-        </is>
+      <c r="AA52" s="2" t="n">
+        <v>46128.06666666667</v>
       </c>
       <c r="AB52" t="inlineStr"/>
       <c r="AC52" t="n">
@@ -6861,10 +6763,8 @@
       <c r="Z53" t="n">
         <v>50724</v>
       </c>
-      <c r="AA53" t="inlineStr">
-        <is>
-          <t>2026-04-16 10:00</t>
-        </is>
+      <c r="AA53" s="2" t="n">
+        <v>46128.41666666666</v>
       </c>
       <c r="AB53" t="inlineStr"/>
       <c r="AC53" t="n">
@@ -6987,10 +6887,8 @@
       <c r="Z54" t="n">
         <v>4627</v>
       </c>
-      <c r="AA54" t="inlineStr">
-        <is>
-          <t>2026-04-16 09:43</t>
-        </is>
+      <c r="AA54" s="2" t="n">
+        <v>46128.40486111111</v>
       </c>
       <c r="AB54" t="inlineStr"/>
       <c r="AC54" t="n">
@@ -7113,10 +7011,8 @@
       <c r="Z55" t="n">
         <v>4623</v>
       </c>
-      <c r="AA55" t="inlineStr">
-        <is>
-          <t>2026-04-16 10:10</t>
-        </is>
+      <c r="AA55" s="2" t="n">
+        <v>46128.42361111111</v>
       </c>
       <c r="AB55" t="inlineStr"/>
       <c r="AC55" t="n">
@@ -7239,10 +7135,8 @@
       <c r="Z56" t="n">
         <v>4620</v>
       </c>
-      <c r="AA56" t="inlineStr">
-        <is>
-          <t>2026-04-16 10:12</t>
-        </is>
+      <c r="AA56" s="2" t="n">
+        <v>46128.425</v>
       </c>
       <c r="AB56" t="inlineStr"/>
       <c r="AC56" t="n">
@@ -7361,10 +7255,8 @@
       <c r="Z57" t="n">
         <v>430</v>
       </c>
-      <c r="AA57" t="inlineStr">
-        <is>
-          <t>2026-04-16 09:41</t>
-        </is>
+      <c r="AA57" s="2" t="n">
+        <v>46128.40347222222</v>
       </c>
       <c r="AB57" t="inlineStr"/>
       <c r="AC57" t="n">
@@ -7483,10 +7375,8 @@
       <c r="Z58" t="n">
         <v>5337.5</v>
       </c>
-      <c r="AA58" t="inlineStr">
-        <is>
-          <t>2026-04-16 12:03</t>
-        </is>
+      <c r="AA58" s="2" t="n">
+        <v>46128.50208333333</v>
       </c>
       <c r="AB58" t="inlineStr"/>
       <c r="AC58" t="n">
@@ -7605,10 +7495,8 @@
       <c r="Z59" t="n">
         <v>765.79</v>
       </c>
-      <c r="AA59" t="inlineStr">
-        <is>
-          <t>2026-04-16 11:32</t>
-        </is>
+      <c r="AA59" s="2" t="n">
+        <v>46128.48055555556</v>
       </c>
       <c r="AB59" t="inlineStr"/>
       <c r="AC59" t="n">
@@ -7723,10 +7611,8 @@
       <c r="Z60" t="n">
         <v>419</v>
       </c>
-      <c r="AA60" t="inlineStr">
-        <is>
-          <t>2026-04-16 19:23</t>
-        </is>
+      <c r="AA60" s="2" t="n">
+        <v>46128.80763888889</v>
       </c>
       <c r="AB60" t="inlineStr"/>
       <c r="AC60" t="n">
@@ -7845,10 +7731,8 @@
       <c r="Z61" t="n">
         <v>1136.71</v>
       </c>
-      <c r="AA61" t="inlineStr">
-        <is>
-          <t>2026-04-16 21:10</t>
-        </is>
+      <c r="AA61" s="2" t="n">
+        <v>46128.88194444445</v>
       </c>
       <c r="AB61" t="inlineStr"/>
       <c r="AC61" t="n">
@@ -7967,10 +7851,8 @@
       <c r="Z62" t="n">
         <v>1012.25</v>
       </c>
-      <c r="AA62" t="inlineStr">
-        <is>
-          <t>2026-04-16 23:18</t>
-        </is>
+      <c r="AA62" s="2" t="n">
+        <v>46128.97083333333</v>
       </c>
       <c r="AB62" t="inlineStr"/>
       <c r="AC62" t="n">
@@ -8093,10 +7975,8 @@
       <c r="Z63" t="n">
         <v>940.4</v>
       </c>
-      <c r="AA63" t="inlineStr">
-        <is>
-          <t>2026-04-17 08:14</t>
-        </is>
+      <c r="AA63" s="2" t="n">
+        <v>46129.34305555555</v>
       </c>
       <c r="AB63" t="inlineStr"/>
       <c r="AC63" t="n">
@@ -8215,10 +8095,8 @@
       <c r="Z64" t="n">
         <v>1188</v>
       </c>
-      <c r="AA64" t="inlineStr">
-        <is>
-          <t>2026-04-17 08:47</t>
-        </is>
+      <c r="AA64" s="2" t="n">
+        <v>46129.36597222222</v>
       </c>
       <c r="AB64" t="inlineStr"/>
       <c r="AC64" t="n">
@@ -8337,10 +8215,8 @@
       <c r="Z65" t="n">
         <v>1188</v>
       </c>
-      <c r="AA65" t="inlineStr">
-        <is>
-          <t>2026-04-17 08:48</t>
-        </is>
+      <c r="AA65" s="2" t="n">
+        <v>46129.36666666667</v>
       </c>
       <c r="AB65" t="inlineStr"/>
       <c r="AC65" t="n">
@@ -8459,10 +8335,8 @@
       <c r="Z66" t="n">
         <v>1188</v>
       </c>
-      <c r="AA66" t="inlineStr">
-        <is>
-          <t>2026-04-17 08:46</t>
-        </is>
+      <c r="AA66" s="2" t="n">
+        <v>46129.36527777778</v>
       </c>
       <c r="AB66" t="inlineStr"/>
       <c r="AC66" t="n">
@@ -8577,10 +8451,8 @@
       <c r="Z67" t="n">
         <v>489</v>
       </c>
-      <c r="AA67" t="inlineStr">
-        <is>
-          <t>2026-04-17 15:41</t>
-        </is>
+      <c r="AA67" s="2" t="n">
+        <v>46129.65347222222</v>
       </c>
       <c r="AB67" t="inlineStr"/>
       <c r="AC67" t="n">
@@ -8699,10 +8571,8 @@
       <c r="Z68" t="n">
         <v>5865</v>
       </c>
-      <c r="AA68" t="inlineStr">
-        <is>
-          <t>2026-04-17 18:34</t>
-        </is>
+      <c r="AA68" s="2" t="n">
+        <v>46129.77361111111</v>
       </c>
       <c r="AB68" t="inlineStr"/>
       <c r="AC68" t="n">
@@ -8817,10 +8687,8 @@
       <c r="Z69" t="n">
         <v>1675.95</v>
       </c>
-      <c r="AA69" t="inlineStr">
-        <is>
-          <t>2026-04-17 19:12</t>
-        </is>
+      <c r="AA69" s="2" t="n">
+        <v>46129.8</v>
       </c>
       <c r="AB69" t="inlineStr"/>
       <c r="AC69" t="n">
@@ -8943,10 +8811,8 @@
       <c r="Z70" t="n">
         <v>4620</v>
       </c>
-      <c r="AA70" t="inlineStr">
-        <is>
-          <t>2026-04-17 18:29</t>
-        </is>
+      <c r="AA70" s="2" t="n">
+        <v>46129.77013888889</v>
       </c>
       <c r="AB70" t="inlineStr"/>
       <c r="AC70" t="n">
@@ -9061,10 +8927,8 @@
       <c r="Z71" t="n">
         <v>2661</v>
       </c>
-      <c r="AA71" t="inlineStr">
-        <is>
-          <t>2026-04-17 18:34</t>
-        </is>
+      <c r="AA71" s="2" t="n">
+        <v>46129.77361111111</v>
       </c>
       <c r="AB71" t="inlineStr"/>
       <c r="AC71" t="n">
@@ -9183,10 +9047,8 @@
       <c r="Z72" t="n">
         <v>5865</v>
       </c>
-      <c r="AA72" t="inlineStr">
-        <is>
-          <t>2026-04-17 18:22</t>
-        </is>
+      <c r="AA72" s="2" t="n">
+        <v>46129.76527777778</v>
       </c>
       <c r="AB72" t="inlineStr"/>
       <c r="AC72" t="n">
@@ -9305,10 +9167,8 @@
       <c r="Z73" t="n">
         <v>5415</v>
       </c>
-      <c r="AA73" t="inlineStr">
-        <is>
-          <t>2026-04-17 18:33</t>
-        </is>
+      <c r="AA73" s="2" t="n">
+        <v>46129.77291666667</v>
       </c>
       <c r="AB73" t="inlineStr"/>
       <c r="AC73" t="n">
@@ -9431,10 +9291,8 @@
       <c r="Z74" t="n">
         <v>10035</v>
       </c>
-      <c r="AA74" t="inlineStr">
-        <is>
-          <t>2026-04-17 18:57</t>
-        </is>
+      <c r="AA74" s="2" t="n">
+        <v>46129.78958333333</v>
       </c>
       <c r="AB74" t="inlineStr"/>
       <c r="AC74" t="n">
@@ -9553,10 +9411,8 @@
       <c r="Z75" t="n">
         <v>10035</v>
       </c>
-      <c r="AA75" t="inlineStr">
-        <is>
-          <t>2026-04-17 18:57</t>
-        </is>
+      <c r="AA75" s="2" t="n">
+        <v>46129.78958333333</v>
       </c>
       <c r="AB75" t="inlineStr"/>
       <c r="AC75" t="n">
@@ -9675,10 +9531,8 @@
       <c r="Z76" t="n">
         <v>5139.75</v>
       </c>
-      <c r="AA76" t="inlineStr">
-        <is>
-          <t>2026-04-17 23:14</t>
-        </is>
+      <c r="AA76" s="2" t="n">
+        <v>46129.96805555555</v>
       </c>
       <c r="AB76" t="inlineStr"/>
       <c r="AC76" t="n">
@@ -9793,10 +9647,8 @@
       <c r="Z77" t="n">
         <v>951</v>
       </c>
-      <c r="AA77" t="inlineStr">
-        <is>
-          <t>2026-04-17 23:37</t>
-        </is>
+      <c r="AA77" s="2" t="n">
+        <v>46129.98402777778</v>
       </c>
       <c r="AB77" t="inlineStr"/>
       <c r="AC77" t="n">
@@ -9915,10 +9767,8 @@
       <c r="Z78" t="n">
         <v>457</v>
       </c>
-      <c r="AA78" t="inlineStr">
-        <is>
-          <t>2026-04-18 16:14</t>
-        </is>
+      <c r="AA78" s="2" t="n">
+        <v>46130.67638888889</v>
       </c>
       <c r="AB78" t="inlineStr"/>
       <c r="AC78" t="n">
@@ -10037,10 +9887,8 @@
       <c r="Z79" t="n">
         <v>179</v>
       </c>
-      <c r="AA79" t="inlineStr">
-        <is>
-          <t>2026-04-18 16:25</t>
-        </is>
+      <c r="AA79" s="2" t="n">
+        <v>46130.68402777778</v>
       </c>
       <c r="AB79" t="inlineStr"/>
       <c r="AC79" t="n">
@@ -10155,10 +10003,8 @@
       <c r="Z80" t="n">
         <v>868</v>
       </c>
-      <c r="AA80" t="inlineStr">
-        <is>
-          <t>2026-04-18 17:57</t>
-        </is>
+      <c r="AA80" s="2" t="n">
+        <v>46130.74791666667</v>
       </c>
       <c r="AB80" t="inlineStr"/>
       <c r="AC80" t="n">
@@ -10277,10 +10123,8 @@
       <c r="Z81" t="n">
         <v>1166</v>
       </c>
-      <c r="AA81" t="inlineStr">
-        <is>
-          <t>2026-04-18 18:44</t>
-        </is>
+      <c r="AA81" s="2" t="n">
+        <v>46130.78055555555</v>
       </c>
       <c r="AB81" t="inlineStr"/>
       <c r="AC81" t="n">
@@ -10399,10 +10243,8 @@
       <c r="Z82" t="n">
         <v>283</v>
       </c>
-      <c r="AA82" t="inlineStr">
-        <is>
-          <t>2026-04-18 20:43</t>
-        </is>
+      <c r="AA82" s="2" t="n">
+        <v>46130.86319444444</v>
       </c>
       <c r="AB82" t="inlineStr"/>
       <c r="AC82" t="n">
@@ -10517,10 +10359,8 @@
       <c r="Z83" t="n">
         <v>2052</v>
       </c>
-      <c r="AA83" t="inlineStr">
-        <is>
-          <t>2026-04-18 21:36</t>
-        </is>
+      <c r="AA83" s="2" t="n">
+        <v>46130.9</v>
       </c>
       <c r="AB83" t="inlineStr"/>
       <c r="AC83" t="n">
@@ -10639,10 +10479,8 @@
       <c r="Z84" t="n">
         <v>6334.1</v>
       </c>
-      <c r="AA84" t="inlineStr">
-        <is>
-          <t>2026-04-18 22:08</t>
-        </is>
+      <c r="AA84" s="2" t="n">
+        <v>46130.92222222222</v>
       </c>
       <c r="AB84" t="inlineStr"/>
       <c r="AC84" t="n">
@@ -10761,10 +10599,8 @@
       <c r="Z85" t="n">
         <v>55835</v>
       </c>
-      <c r="AA85" t="inlineStr">
-        <is>
-          <t>2026-04-19 20:57</t>
-        </is>
+      <c r="AA85" s="2" t="n">
+        <v>46131.87291666667</v>
       </c>
       <c r="AB85" t="inlineStr"/>
       <c r="AC85" t="n">
@@ -10879,10 +10715,8 @@
       <c r="Z86" t="n">
         <v>5524</v>
       </c>
-      <c r="AA86" t="inlineStr">
-        <is>
-          <t>2026-04-19 22:33</t>
-        </is>
+      <c r="AA86" s="2" t="n">
+        <v>46131.93958333333</v>
       </c>
       <c r="AB86" t="inlineStr"/>
       <c r="AC86" t="n">
@@ -10997,10 +10831,8 @@
       <c r="Z87" t="n">
         <v>3344</v>
       </c>
-      <c r="AA87" t="inlineStr">
-        <is>
-          <t>2026-04-20 09:01</t>
-        </is>
+      <c r="AA87" s="2" t="n">
+        <v>46132.37569444445</v>
       </c>
       <c r="AB87" t="inlineStr"/>
       <c r="AC87" t="n">
@@ -11119,10 +10951,8 @@
       <c r="Z88" t="n">
         <v>1545</v>
       </c>
-      <c r="AA88" t="inlineStr">
-        <is>
-          <t>2026-04-20 12:04</t>
-        </is>
+      <c r="AA88" s="2" t="n">
+        <v>46132.50277777778</v>
       </c>
       <c r="AB88" t="inlineStr"/>
       <c r="AC88" t="n">
@@ -11237,10 +11067,8 @@
       <c r="Z89" t="n">
         <v>664.9400000000001</v>
       </c>
-      <c r="AA89" t="inlineStr">
-        <is>
-          <t>2026-04-20 12:16</t>
-        </is>
+      <c r="AA89" s="2" t="n">
+        <v>46132.51111111111</v>
       </c>
       <c r="AB89" t="inlineStr"/>
       <c r="AC89" t="n">
@@ -11355,10 +11183,8 @@
       <c r="Z90" t="n">
         <v>232</v>
       </c>
-      <c r="AA90" t="inlineStr">
-        <is>
-          <t>2026-04-20 13:33</t>
-        </is>
+      <c r="AA90" s="2" t="n">
+        <v>46132.56458333333</v>
       </c>
       <c r="AB90" t="inlineStr"/>
       <c r="AC90" t="n">
@@ -11481,10 +11307,8 @@
       <c r="Z91" t="n">
         <v>743</v>
       </c>
-      <c r="AA91" t="inlineStr">
-        <is>
-          <t>2026-04-20 14:35</t>
-        </is>
+      <c r="AA91" s="2" t="n">
+        <v>46132.60763888889</v>
       </c>
       <c r="AB91" t="inlineStr"/>
       <c r="AC91" t="n">
@@ -11607,10 +11431,8 @@
       <c r="Z92" t="n">
         <v>743</v>
       </c>
-      <c r="AA92" t="inlineStr">
-        <is>
-          <t>2026-04-20 14:35</t>
-        </is>
+      <c r="AA92" s="2" t="n">
+        <v>46132.60763888889</v>
       </c>
       <c r="AB92" t="inlineStr"/>
       <c r="AC92" t="n">
@@ -11725,10 +11547,8 @@
       <c r="Z93" t="n">
         <v>3166</v>
       </c>
-      <c r="AA93" t="inlineStr">
-        <is>
-          <t>2026-04-20 14:58</t>
-        </is>
+      <c r="AA93" s="2" t="n">
+        <v>46132.62361111111</v>
       </c>
       <c r="AB93" t="inlineStr"/>
       <c r="AC93" t="n">
@@ -11843,10 +11663,8 @@
       <c r="Z94" t="n">
         <v>3308</v>
       </c>
-      <c r="AA94" t="inlineStr">
-        <is>
-          <t>2026-04-20 14:58</t>
-        </is>
+      <c r="AA94" s="2" t="n">
+        <v>46132.62361111111</v>
       </c>
       <c r="AB94" t="inlineStr"/>
       <c r="AC94" t="n">
@@ -11961,10 +11779,8 @@
       <c r="Z95" t="n">
         <v>941</v>
       </c>
-      <c r="AA95" t="inlineStr">
-        <is>
-          <t>2026-04-20 16:48</t>
-        </is>
+      <c r="AA95" s="2" t="n">
+        <v>46132.7</v>
       </c>
       <c r="AB95" t="inlineStr"/>
       <c r="AC95" t="n">
@@ -12079,10 +11895,8 @@
       <c r="Z96" t="n">
         <v>4047</v>
       </c>
-      <c r="AA96" t="inlineStr">
-        <is>
-          <t>2026-04-20 18:22</t>
-        </is>
+      <c r="AA96" s="2" t="n">
+        <v>46132.76527777778</v>
       </c>
       <c r="AB96" t="inlineStr"/>
       <c r="AC96" t="n">
@@ -12201,10 +12015,8 @@
       <c r="Z97" t="n">
         <v>761</v>
       </c>
-      <c r="AA97" t="inlineStr">
-        <is>
-          <t>2026-04-20 20:31</t>
-        </is>
+      <c r="AA97" s="2" t="n">
+        <v>46132.85486111111</v>
       </c>
       <c r="AB97" t="inlineStr"/>
       <c r="AC97" t="n">
@@ -12319,10 +12131,8 @@
       <c r="Z98" t="n">
         <v>425</v>
       </c>
-      <c r="AA98" t="inlineStr">
-        <is>
-          <t>2026-04-21 00:28</t>
-        </is>
+      <c r="AA98" s="2" t="n">
+        <v>46133.01944444444</v>
       </c>
       <c r="AB98" t="inlineStr"/>
       <c r="AC98" t="n">
@@ -12437,10 +12247,8 @@
       <c r="Z99" t="n">
         <v>5465</v>
       </c>
-      <c r="AA99" t="inlineStr">
-        <is>
-          <t>2026-04-21 08:18</t>
-        </is>
+      <c r="AA99" s="2" t="n">
+        <v>46133.34583333333</v>
       </c>
       <c r="AB99" t="inlineStr"/>
       <c r="AC99" t="n">
@@ -12555,10 +12363,8 @@
       <c r="Z100" t="n">
         <v>42138</v>
       </c>
-      <c r="AA100" t="inlineStr">
-        <is>
-          <t>2026-04-21 11:43</t>
-        </is>
+      <c r="AA100" s="2" t="n">
+        <v>46133.48819444444</v>
       </c>
       <c r="AB100" t="inlineStr"/>
       <c r="AC100" t="n">
@@ -12673,10 +12479,8 @@
       <c r="Z101" t="n">
         <v>976</v>
       </c>
-      <c r="AA101" t="inlineStr">
-        <is>
-          <t>2026-04-21 16:59</t>
-        </is>
+      <c r="AA101" s="2" t="n">
+        <v>46133.70763888889</v>
       </c>
       <c r="AB101" t="inlineStr"/>
       <c r="AC101" t="n">
@@ -12795,10 +12599,8 @@
       <c r="Z102" t="n">
         <v>1109</v>
       </c>
-      <c r="AA102" t="inlineStr">
-        <is>
-          <t>2026-04-21 19:59</t>
-        </is>
+      <c r="AA102" s="2" t="n">
+        <v>46133.83263888889</v>
       </c>
       <c r="AB102" t="inlineStr"/>
       <c r="AC102" t="n">
@@ -12918,10 +12720,8 @@
       <c r="Z103" t="n">
         <v>2362</v>
       </c>
-      <c r="AA103" t="inlineStr">
-        <is>
-          <t>2026-04-21 19:46</t>
-        </is>
+      <c r="AA103" s="2" t="n">
+        <v>46133.82361111111</v>
       </c>
       <c r="AB103" t="inlineStr"/>
       <c r="AC103" t="n">
@@ -13040,10 +12840,8 @@
       <c r="Z104" t="n">
         <v>1099</v>
       </c>
-      <c r="AA104" t="inlineStr">
-        <is>
-          <t>2026-04-21 21:37</t>
-        </is>
+      <c r="AA104" s="2" t="n">
+        <v>46133.90069444444</v>
       </c>
       <c r="AB104" t="inlineStr"/>
       <c r="AC104" t="n">
@@ -13162,10 +12960,8 @@
       <c r="Z105" t="n">
         <v>11980</v>
       </c>
-      <c r="AA105" t="inlineStr">
-        <is>
-          <t>2026-04-21 21:00</t>
-        </is>
+      <c r="AA105" s="2" t="n">
+        <v>46133.875</v>
       </c>
       <c r="AB105" t="inlineStr"/>
       <c r="AC105" t="n">
@@ -13280,10 +13076,8 @@
       <c r="Z106" t="n">
         <v>768</v>
       </c>
-      <c r="AA106" t="inlineStr">
-        <is>
-          <t>2026-04-22 08:51</t>
-        </is>
+      <c r="AA106" s="2" t="n">
+        <v>46134.36875</v>
       </c>
       <c r="AB106" t="inlineStr"/>
       <c r="AC106" t="n">
@@ -13406,10 +13200,8 @@
       <c r="Z107" t="n">
         <v>899</v>
       </c>
-      <c r="AA107" t="inlineStr">
-        <is>
-          <t>2026-04-22 11:20</t>
-        </is>
+      <c r="AA107" s="2" t="n">
+        <v>46134.47222222222</v>
       </c>
       <c r="AB107" t="inlineStr"/>
       <c r="AC107" t="n">
@@ -13524,10 +13316,8 @@
       <c r="Z108" t="n">
         <v>4500.3</v>
       </c>
-      <c r="AA108" t="inlineStr">
-        <is>
-          <t>2026-04-22 15:50</t>
-        </is>
+      <c r="AA108" s="2" t="n">
+        <v>46134.65972222222</v>
       </c>
       <c r="AB108" t="inlineStr"/>
       <c r="AC108" t="n">
@@ -13642,10 +13432,8 @@
       <c r="Z109" t="n">
         <v>2703.41</v>
       </c>
-      <c r="AA109" t="inlineStr">
-        <is>
-          <t>2026-04-22 21:04</t>
-        </is>
+      <c r="AA109" s="2" t="n">
+        <v>46134.87777777778</v>
       </c>
       <c r="AB109" t="inlineStr"/>
       <c r="AC109" t="n">
@@ -13760,10 +13548,8 @@
       <c r="Z110" t="n">
         <v>749</v>
       </c>
-      <c r="AA110" t="inlineStr">
-        <is>
-          <t>2026-04-23 00:46</t>
-        </is>
+      <c r="AA110" s="2" t="n">
+        <v>46135.03194444445</v>
       </c>
       <c r="AB110" t="inlineStr"/>
       <c r="AC110" t="n">
@@ -13878,10 +13664,8 @@
       <c r="Z111" t="n">
         <v>2038</v>
       </c>
-      <c r="AA111" t="inlineStr">
-        <is>
-          <t>2026-04-23 07:18</t>
-        </is>
+      <c r="AA111" s="2" t="n">
+        <v>46135.30416666667</v>
       </c>
       <c r="AB111" t="inlineStr"/>
       <c r="AC111" t="n">

</xml_diff>